<commit_message>
Actualiza datos y modelo financiero por decisiones del director
- Nombres: Guido Maldonado (era Mardonado), Fabelly Maciel Fabian Bello (era Fabelle).
- La Vega: Leticia González confirmada (1 asesor). SD: Marleny + Sandrita confirmados.
- Modelo financiero (estado.json + build_finanzas/docx/drive):
  - Piso: completar 100 personas en la casa (≈47 operativos + ~53 participantes).
  - Meta de recaudación = COSTO TOTAL (≈$533,481), no un número fijo inventado.
    Se cubre con cuotas (participantes $3,000 + equipo $1,500–2,000) + rifa/venta de
    comida + donaciones (montos VARIABLES, lo que se recaude).
  - Quitadas las cifras inventadas (meta $260K, rifa $130K, profondo2/donaciones $50K).
    La brecha ($292,231) se calcula = costo − cuotas y la cubre la recaudación variable.
- verify.py: meta ya no exige [PROPUESTA]; blinda contra el viejo $260K.
- Guión 4-jun y banderas actualizados. TODO PASS.

https://claude.ai/code/session_016scja59CycFFrqKgYsUPWh
</commit_message>
<xml_diff>
--- a/Equipo_ETC88.xlsx
+++ b/Equipo_ETC88.xlsx
@@ -2611,7 +2611,7 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Fabelle maciel fabian bello</t>
+          <t>Fabelly Maciel Fabian Bello</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
@@ -2685,7 +2685,7 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Guido Mardonado</t>
+          <t>Guido Maldonado</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
@@ -5888,7 +5888,7 @@
     <row r="29">
       <c r="A29" s="20" t="inlineStr">
         <is>
-          <t>Fabelle maciel fabian bello</t>
+          <t>Fabelly Maciel Fabian Bello</t>
         </is>
       </c>
       <c r="B29" s="20" t="inlineStr">
@@ -5936,7 +5936,7 @@
     <row r="30">
       <c r="A30" s="20" t="inlineStr">
         <is>
-          <t>Guido Mardonado</t>
+          <t>Guido Maldonado</t>
         </is>
       </c>
       <c r="B30" s="20" t="inlineStr">

</xml_diff>